<commit_message>
resolution de bug de contour
</commit_message>
<xml_diff>
--- a/Projet-Exemple/Generate Files/Bill of Materials/243-TGE-Template.xlsx
+++ b/Projet-Exemple/Generate Files/Bill of Materials/243-TGE-Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2357758\Desktop\Lab1-clickboard\Projet-Exemple\Generate Files\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A3996FF-D034-44F2-8E1B-6BCE9F1F9974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9923513E-E5B6-41F8-96FD-A0F6A6BAE29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{696B8CEC-6B16-4AA9-B3C6-D74CF55BED3E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B1A1B3FD-0C6D-4490-950D-21012B5F9884}"/>
   </bookViews>
   <sheets>
     <sheet name="243-TGE-Template" sheetId="1" r:id="rId1"/>
@@ -92,7 +92,7 @@
     <t>CAP CER 100nF 50V 0402</t>
   </si>
   <si>
-    <t>C1, C2, C3, C4</t>
+    <t>C1, C2, C3, C4, C5</t>
   </si>
   <si>
     <t>Capacitor type 1</t>
@@ -689,7 +689,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39A3BCA-8713-4235-95CD-67C2DD9C0544}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F03AA4F-0543-428E-B828-B4D745075093}">
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -758,7 +758,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
ajout de nom et port io et mux
</commit_message>
<xml_diff>
--- a/Projet-Exemple/Generate Files/Bill of Materials/243-TGE-Template.xlsx
+++ b/Projet-Exemple/Generate Files/Bill of Materials/243-TGE-Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2357758\Desktop\Lab1-clickboard\Projet-Exemple\Generate Files\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9923513E-E5B6-41F8-96FD-A0F6A6BAE29C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C60B098-4EAB-4FDD-B681-849F528BC276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B1A1B3FD-0C6D-4490-950D-21012B5F9884}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63E50BB6-7737-46F8-BC4F-DFAC74B01252}"/>
   </bookViews>
   <sheets>
     <sheet name="243-TGE-Template" sheetId="1" r:id="rId1"/>
@@ -689,7 +689,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F03AA4F-0543-428E-B828-B4D745075093}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2169D65E-CB8C-4666-AC4E-0B703DFBCDDD}">
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
ajustement des pieces 0603
</commit_message>
<xml_diff>
--- a/Projet-Exemple/Generate Files/Bill of Materials/243-TGE-Template.xlsx
+++ b/Projet-Exemple/Generate Files/Bill of Materials/243-TGE-Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2357758\Desktop\Lab1-clickboard\Projet-Exemple\Generate Files\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C60B098-4EAB-4FDD-B681-849F528BC276}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{305069B8-FD86-4CE6-BB6C-D5649EF18165}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{63E50BB6-7737-46F8-BC4F-DFAC74B01252}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E4BF0D22-4294-46D2-9A17-ED0F5EF70975}"/>
   </bookViews>
   <sheets>
     <sheet name="243-TGE-Template" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="84">
   <si>
     <t>Code CEGEP</t>
   </si>
@@ -83,13 +83,13 @@
     <t>Supplier Part Number 2</t>
   </si>
   <si>
-    <t>KCOND01SM</t>
-  </si>
-  <si>
-    <t>CAP001</t>
-  </si>
-  <si>
-    <t>CAP CER 100nF 50V 0402</t>
+    <t>COND0143SM</t>
+  </si>
+  <si>
+    <t>CAP002</t>
+  </si>
+  <si>
+    <t>CAP CER 100nF 50V 0603</t>
   </si>
   <si>
     <t>C1, C2, C3, C4, C5</t>
@@ -101,13 +101,31 @@
     <t>Yageo</t>
   </si>
   <si>
-    <t>CC0402KRX7R9BB104</t>
+    <t>CC0603KRX7R9BB104</t>
   </si>
   <si>
     <t>LCSC</t>
   </si>
   <si>
-    <t>C131394</t>
+    <t>C14663</t>
+  </si>
+  <si>
+    <t>CAP022</t>
+  </si>
+  <si>
+    <t>CAP CER 2.2uF 10V X7R 0603</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
+    <t>CL10B225KP8NNNC</t>
+  </si>
+  <si>
+    <t>C100082</t>
   </si>
   <si>
     <t/>
@@ -155,25 +173,22 @@
     <t>SAM9303-ND</t>
   </si>
   <si>
-    <t>RES1KSM</t>
-  </si>
-  <si>
-    <t>RES006</t>
-  </si>
-  <si>
-    <t>Res 1k 1% 0402</t>
-  </si>
-  <si>
-    <t>R1, R2</t>
+    <t>RES015</t>
+  </si>
+  <si>
+    <t>Res 1k 1% 0603</t>
+  </si>
+  <si>
+    <t>R1, R2, R5, R6, R7, R8, R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R20</t>
   </si>
   <si>
     <t>Resistor type 1</t>
   </si>
   <si>
-    <t>RC0402FR-071kL</t>
-  </si>
-  <si>
-    <t>C106235</t>
+    <t>RC0603FR-071KL</t>
+  </si>
+  <si>
+    <t>C22548</t>
   </si>
   <si>
     <t>RESI0238-0603</t>
@@ -192,21 +207,6 @@
   </si>
   <si>
     <t>C98220</t>
-  </si>
-  <si>
-    <t>RES029</t>
-  </si>
-  <si>
-    <t>Res 100R 1% 0603</t>
-  </si>
-  <si>
-    <t>R5, R6, R7, R8, R9, R10, R11, R12, R13, R14, R15, R16, R17, R18, R19, R20</t>
-  </si>
-  <si>
-    <t>RC0603FR-07100RL</t>
-  </si>
-  <si>
-    <t>C105588</t>
   </si>
   <si>
     <t>SW_DIP_50MIL_4POS</t>
@@ -689,7 +689,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2169D65E-CB8C-4666-AC4E-0B703DFBCDDD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A35DF7F9-1E60-4847-B43B-770D5E492150}">
   <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -782,159 +782,157 @@
       <c r="M2" s="1"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="1">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>20</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="E4" s="1">
         <v>2</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="L4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M4" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="E5" s="1">
         <v>2</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="I5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="L5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="1">
+        <v>18</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="E6" s="1">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>20</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
+      <c r="A7" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="B7" s="1"/>
       <c r="C7" s="2" t="s">
         <v>50</v>
@@ -943,13 +941,13 @@
         <v>51</v>
       </c>
       <c r="E7" s="1">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>52</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>18</v>
@@ -1034,7 +1032,7 @@
         <v>67</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="M9" s="2" t="s">
         <v>68</v>
@@ -1071,7 +1069,7 @@
         <v>74</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="M10" s="2" t="s">
         <v>75</v>

</xml_diff>